<commit_message>
Initial commit Updated Code
</commit_message>
<xml_diff>
--- a/sample_teams_players.xlsx
+++ b/sample_teams_players.xlsx
@@ -417,11 +417,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -435,6 +436,11 @@
           <t>Player</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -447,6 +453,11 @@
           <t>Team A Player 1</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -459,6 +470,7 @@
           <t>Team A Player 2</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -471,6 +483,7 @@
           <t>Team A Player 3</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -483,6 +496,7 @@
           <t>Team A Player 4</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -495,6 +509,7 @@
           <t>Team A Player 5</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -507,6 +522,7 @@
           <t>Team A Player 6</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -519,6 +535,7 @@
           <t>Team A Player 7</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -531,6 +548,7 @@
           <t>Team A Player 8</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -543,6 +561,7 @@
           <t>Team A Player 9</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -555,6 +574,7 @@
           <t>Team A Player 10</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -567,6 +587,7 @@
           <t>Team A Player 11</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -579,6 +600,11 @@
           <t>Team B Player 1</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -591,6 +617,7 @@
           <t>Team B Player 2</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -603,6 +630,7 @@
           <t>Team B Player 3</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -615,6 +643,7 @@
           <t>Team B Player 4</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -627,6 +656,7 @@
           <t>Team B Player 5</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -639,6 +669,7 @@
           <t>Team B Player 6</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -651,6 +682,7 @@
           <t>Team B Player 7</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -663,6 +695,7 @@
           <t>Team B Player 8</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -675,6 +708,7 @@
           <t>Team B Player 9</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -687,6 +721,7 @@
           <t>Team B Player 10</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -699,6 +734,7 @@
           <t>Team B Player 11</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>